<commit_message>
Paramount,Google and Doordash update
</commit_message>
<xml_diff>
--- a/003_SapAriba_Shell_Performer/lib/net45/Data/Config.xlsx
+++ b/003_SapAriba_Shell_Performer/lib/net45/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grmusarpadev10\Desktop\Git_Upload_Sap\grm-usa-ar-ariba-performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NA-Automation\Git Repo\grm-usa-ar-ariba-performer\003_SapAriba_Shell_Performer\lib\net45\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D70B89-69D8-4678-A258-EE46FF02D900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90960F3-D5DA-482D-B24F-5916FF55C99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="10815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13425" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="141">
   <si>
     <t>Name</t>
   </si>
@@ -458,6 +458,9 @@
   </si>
   <si>
     <t>When testTesting is true invoices are not submitted</t>
+  </si>
+  <si>
+    <t>AribaSupplierUrl</t>
   </si>
 </sst>
 </file>
@@ -990,35 +993,32 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="23">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1026,14 +1026,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="59">
     <cellStyle name="Comma 2" xfId="38" xr:uid="{B0A0F9FC-9ADB-4FDF-AD5C-0A7345AEB1BA}"/>
@@ -1110,9 +1107,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1150,7 +1147,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1256,7 +1253,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1398,7 +1395,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1416,38 +1413,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" s="8" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6"/>
+      <c r="Z1" s="6"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1495,7 +1492,7 @@
       <c r="A8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="14" t="s">
         <v>129</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1593,18 +1590,18 @@
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="16" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="16" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2736,10 +2733,10 @@
       <c r="A13" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2747,19 +2744,18 @@
       <c r="A14" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="C14" s="15"/>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="17" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2781,7 +2777,7 @@
       <c r="A18" t="s">
         <v>107</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2789,7 +2785,7 @@
       <c r="A19" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3825,7 +3821,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
         <v>31</v>
@@ -3902,7 +3898,7 @@
       <c r="A11" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D11" t="s">
@@ -3913,7 +3909,7 @@
       <c r="A12" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="19" t="s">
         <v>118</v>
       </c>
       <c r="D12" t="s">
@@ -3946,7 +3942,7 @@
       <c r="A15" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="18" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3954,97 +3950,97 @@
       <c r="A16" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="18" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24" t="s">
+      <c r="C17" s="20"/>
+      <c r="D17" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="12" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24" t="s">
+      <c r="C18" s="20"/>
+      <c r="D18" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="12" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24" t="s">
+      <c r="C19" s="20"/>
+      <c r="D19" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="12" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24" t="s">
+      <c r="C20" s="20"/>
+      <c r="D20" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="12" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24" t="s">
+      <c r="C21" s="20"/>
+      <c r="D21" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="12" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24" t="s">
+      <c r="C22" s="20"/>
+      <c r="D22" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -5046,115 +5042,115 @@
   <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.7109375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="98" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="64" style="13" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="13"/>
+    <col min="1" max="1" width="21.7109375" style="12" customWidth="1"/>
+    <col min="2" max="2" width="98" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64" style="12" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="12" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:26" s="11" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
     </row>
     <row r="3" spans="1:26">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="12" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:26">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="30">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="22" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="30">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="22" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:26">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:26">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:26">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="12" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:26">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>127</v>
       </c>
     </row>
@@ -5240,10 +5236,10 @@
       </c>
     </row>
     <row r="7" spans="1:26">
-      <c r="A7" s="27" t="s">
+      <c r="A7" t="s">
         <v>137</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="2" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>